<commit_message>
fix: align extracts with verified header contract
</commit_message>
<xml_diff>
--- a/synthetic_library/config/config_field_map.xlsx
+++ b/synthetic_library/config/config_field_map.xlsx
@@ -443,12 +443,12 @@
   <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -798,7 +798,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>FBS LoB</t>
+          <t>FBS Line of Business</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -821,7 +821,11 @@
           <t>confirmed</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>header verified against real report — 'FBS LoB' shorthand is dead</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -851,7 +855,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Line Manager to be ADDED to real position report</t>
+          <t>Line Manager Name absent from today's real position report — must be ADDED to the purpose-built report</t>
         </is>
       </c>
     </row>
@@ -883,7 +887,7 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>semantics unconfirmed — do not compare</t>
+          <t>both columns exist in the real reports; SEMANTICS unconfirmed — do not compare (synthetic values deliberately differ in form)</t>
         </is>
       </c>
     </row>
@@ -915,7 +919,7 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>in NEITHER current report — add to both purpose-built reports</t>
+          <t>in NEITHER real report — add to both purpose-built reports</t>
         </is>
       </c>
     </row>

</xml_diff>